<commit_message>
changes df.columns = [c.strip() for c in df.columns] to df = df.loc[:, ~df.columns.str.contains(^Unnamed, na=False)] in app.py
</commit_message>
<xml_diff>
--- a/data/raw/town_scores.xlsx
+++ b/data/raw/town_scores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/russ_the_bus/Desktop/Bubble_Move_Meter/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC101A9-4F03-9448-98EF-5C1F7D90151B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012B9334-CBE8-8347-A57D-BA630F1FBA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{11A6349F-FCD6-4A46-9216-B6FF8C3D0BBE}"/>
   </bookViews>
@@ -151,8 +151,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="00000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -207,15 +207,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,27 +553,27 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="6.5" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -589,67 +588,67 @@
       <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="S1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="V1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="W1" s="7" t="s">
+      <c r="W1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="7"/>
+      <c r="Z1" s="5"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -658,67 +657,67 @@
       <c r="B2" s="1">
         <v>2459</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="6">
         <v>85</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="6">
         <v>1650000</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="6">
         <v>0.124</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>624.32000000000005</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="6">
         <v>96</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="6">
         <v>92</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="6">
         <v>61</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="6">
         <v>68</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="6">
         <v>70</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="6">
         <v>45</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="6">
         <v>35</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q2">
+      <c r="Q2" s="6">
         <v>75</v>
       </c>
-      <c r="R2" s="3">
+      <c r="R2" s="6">
         <v>210.79</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="6">
         <v>0.05</v>
       </c>
-      <c r="T2">
+      <c r="T2" s="6">
         <v>46</v>
       </c>
-      <c r="U2">
+      <c r="U2" s="6">
         <v>88</v>
       </c>
-      <c r="V2" s="2">
+      <c r="V2" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W2">
+      <c r="W2" s="6">
         <v>63</v>
       </c>
     </row>
@@ -729,67 +728,67 @@
       <c r="B3" s="1">
         <v>2451</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="6">
         <v>83</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="6">
         <v>680100</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="6">
         <v>7.8E-2</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>352.42</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="6">
         <v>81</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="6">
         <v>77</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="6">
         <v>59</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="6">
         <v>67</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="6">
         <v>63</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="6">
         <v>54</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="6">
         <v>38</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="6">
         <v>74</v>
       </c>
-      <c r="R3" s="3">
+      <c r="R3" s="6">
         <v>117.93</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="6">
         <v>0.05</v>
       </c>
-      <c r="T3">
+      <c r="T3" s="6">
         <v>50</v>
       </c>
-      <c r="U3">
+      <c r="U3" s="6">
         <v>68</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W3">
+      <c r="W3" s="6">
         <v>54</v>
       </c>
     </row>
@@ -800,67 +799,67 @@
       <c r="B4" s="1">
         <v>2452</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="6">
         <v>81</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="6">
         <v>788400</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="6">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>402.76</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="6">
         <v>83</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="6">
         <v>77</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="6">
         <v>60</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="6">
         <v>68</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="6">
         <v>59</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="6">
         <v>36</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="6">
         <v>33</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="6">
         <v>74</v>
       </c>
-      <c r="R4" s="3">
+      <c r="R4" s="6">
         <v>106.67</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="6">
         <v>0.05</v>
       </c>
-      <c r="T4">
+      <c r="T4" s="6">
         <v>51</v>
       </c>
-      <c r="U4">
+      <c r="U4" s="6">
         <v>73</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W4">
+      <c r="W4" s="6">
         <v>54</v>
       </c>
     </row>
@@ -871,67 +870,67 @@
       <c r="B5" s="1">
         <v>2453</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="6">
         <v>87</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="6">
         <v>703500</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="6">
         <v>0.08</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>350.02</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="6">
         <v>80</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="6">
         <v>77</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="6">
         <v>60</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="6">
         <v>63</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="6">
         <v>69</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="6">
         <v>60</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="6">
         <v>66</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="6">
         <v>80</v>
       </c>
-      <c r="R5" s="3">
+      <c r="R5" s="6">
         <v>111.29</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="6">
         <v>0.05</v>
       </c>
-      <c r="T5">
+      <c r="T5" s="6">
         <v>48</v>
       </c>
-      <c r="U5">
+      <c r="U5" s="6">
         <v>66</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W5">
+      <c r="W5" s="6">
         <v>52</v>
       </c>
     </row>
@@ -942,67 +941,67 @@
       <c r="B6" s="1">
         <v>1890</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="6">
         <v>84</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="6">
         <v>1480000</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="6">
         <v>9.3000000000000013E-2</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="6">
         <v>545.66999999999996</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="6">
         <v>96</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="6">
         <v>81</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="6">
         <v>59</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="6">
         <v>67</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="6">
         <v>68</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="6">
         <v>44</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="6">
         <v>36</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q6">
+      <c r="Q6" s="6">
         <v>79</v>
       </c>
-      <c r="R6" s="3">
+      <c r="R6" s="6">
         <v>208.53</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="6">
         <v>0.05</v>
       </c>
-      <c r="T6">
+      <c r="T6" s="6">
         <v>42</v>
       </c>
-      <c r="U6">
+      <c r="U6" s="6">
         <v>77</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W6">
+      <c r="W6" s="6">
         <v>61</v>
       </c>
     </row>
@@ -1013,67 +1012,67 @@
       <c r="B7" s="1">
         <v>2461</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="6">
         <v>84</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="6">
         <v>1320000</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="6">
         <v>0.12</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="6">
         <v>580.05999999999995</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>96</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="6">
         <v>80</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="6">
         <v>60</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="6">
         <v>65</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="6">
         <v>79</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="6">
         <v>35</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="6">
         <v>22</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="6">
         <v>82</v>
       </c>
-      <c r="R7" s="3">
+      <c r="R7" s="6">
         <v>191.71</v>
       </c>
-      <c r="S7" s="2">
+      <c r="S7" s="6">
         <v>0.05</v>
       </c>
-      <c r="T7">
+      <c r="T7" s="6">
         <v>50</v>
       </c>
-      <c r="U7">
+      <c r="U7" s="6">
         <v>83</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W7">
+      <c r="W7" s="6">
         <v>66</v>
       </c>
     </row>
@@ -1084,67 +1083,67 @@
       <c r="B8" s="1">
         <v>2464</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="6">
         <v>81</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="6">
         <v>895200</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="6">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="6">
         <v>203.66</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="6">
         <v>91</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="6">
         <v>75</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="6">
         <v>60</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="6">
         <v>65</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="6">
         <v>70</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="6">
         <v>34</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="6">
         <v>22</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="6">
         <v>71</v>
       </c>
-      <c r="R8" s="3">
+      <c r="R8" s="6">
         <v>126.35</v>
       </c>
-      <c r="S8" s="2">
+      <c r="S8" s="6">
         <v>0.05</v>
       </c>
-      <c r="T8">
+      <c r="T8" s="6">
         <v>42</v>
       </c>
-      <c r="U8">
+      <c r="U8" s="6">
         <v>72</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W8">
+      <c r="W8" s="6">
         <v>66</v>
       </c>
     </row>
@@ -1155,67 +1154,67 @@
       <c r="B9" s="1">
         <v>2460</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="6">
         <v>81</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="6">
         <v>1150000</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="6">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="6">
         <v>436.07</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="6">
         <v>96</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="6">
         <v>76</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="6">
         <v>62</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="6">
         <v>65</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="6">
         <v>69</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="6">
         <v>35</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="6">
         <v>21</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="6">
         <v>73</v>
       </c>
-      <c r="R9" s="3">
+      <c r="R9" s="6">
         <v>149</v>
       </c>
-      <c r="S9" s="2">
+      <c r="S9" s="6">
         <v>0.05</v>
       </c>
-      <c r="T9">
+      <c r="T9" s="6">
         <v>46</v>
       </c>
-      <c r="U9">
+      <c r="U9" s="6">
         <v>79</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W9">
+      <c r="W9" s="6">
         <v>58</v>
       </c>
     </row>
@@ -1226,67 +1225,67 @@
       <c r="B10" s="1">
         <v>2465</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="6">
         <v>82</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="6">
         <v>1250000</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="6">
         <v>9.1999999999999998E-3</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="6">
         <v>9.1999999999999998E-2</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="6">
         <v>506.85</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="6">
         <v>96</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="6">
         <v>76</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="6">
         <v>61</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="6">
         <v>61</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="6">
         <v>67</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="6">
         <v>31</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="6">
         <v>20</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="6">
         <v>82</v>
       </c>
-      <c r="R10" s="3">
+      <c r="R10" s="6">
         <v>178.33</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="6">
         <v>0.05</v>
       </c>
-      <c r="T10">
+      <c r="T10" s="6">
         <v>47</v>
       </c>
-      <c r="U10">
+      <c r="U10" s="6">
         <v>84</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W10">
+      <c r="W10" s="6">
         <v>58</v>
       </c>
     </row>
@@ -1297,67 +1296,67 @@
       <c r="B11" s="1">
         <v>2466</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="6">
         <v>81</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="6">
         <v>1170000</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="6">
         <v>0.10400000000000001</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="6">
         <v>410.57</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="6">
         <v>96</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="6">
         <v>78</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="6">
         <v>59</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="6">
         <v>60</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="6">
         <v>72</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="6">
         <v>32</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="6">
         <v>19</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="6">
         <v>72</v>
       </c>
-      <c r="R11" s="3">
+      <c r="R11" s="6">
         <v>144.93</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="6">
         <v>0.05</v>
       </c>
-      <c r="T11">
+      <c r="T11" s="6">
         <v>49</v>
       </c>
-      <c r="U11">
+      <c r="U11" s="6">
         <v>80</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W11">
+      <c r="W11" s="6">
         <v>51</v>
       </c>
     </row>
@@ -1368,67 +1367,67 @@
       <c r="B12" s="1">
         <v>2462</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="6">
         <v>81</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="6">
         <v>1320000</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="6">
         <v>0.153</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="6">
         <v>705.81</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="6">
         <v>96</v>
       </c>
-      <c r="I12">
+      <c r="I12" s="6">
         <v>74</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="6">
         <v>57</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="6">
         <v>62</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="6">
         <v>71</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="6">
         <v>22</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="6">
         <v>12</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="6">
         <v>81</v>
       </c>
-      <c r="R12" s="3">
+      <c r="R12" s="6">
         <v>136.38</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="6">
         <v>0.05</v>
       </c>
-      <c r="T12">
+      <c r="T12" s="6">
         <v>45</v>
       </c>
-      <c r="U12">
+      <c r="U12" s="6">
         <v>73</v>
       </c>
-      <c r="V12" s="2">
+      <c r="V12" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W12">
+      <c r="W12" s="6">
         <v>54</v>
       </c>
     </row>
@@ -1439,67 +1438,67 @@
       <c r="B13" s="1">
         <v>2468</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="6">
         <v>81</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="6">
         <v>1850000</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="6">
         <v>0.11199999999999999</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="6">
         <v>591.79</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="6">
         <v>96</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="6">
         <v>81</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="6">
         <v>60</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="6">
         <v>65</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="6">
         <v>70</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="6">
         <v>24</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="6">
         <v>13</v>
       </c>
-      <c r="O13" s="2">
+      <c r="O13" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q13">
+      <c r="Q13" s="6">
         <v>80</v>
       </c>
-      <c r="R13" s="3">
+      <c r="R13" s="6">
         <v>250</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="6">
         <v>0.05</v>
       </c>
-      <c r="T13">
+      <c r="T13" s="6">
         <v>45</v>
       </c>
-      <c r="U13">
+      <c r="U13" s="6">
         <v>90</v>
       </c>
-      <c r="V13" s="2">
+      <c r="V13" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W13">
+      <c r="W13" s="6">
         <v>62</v>
       </c>
     </row>
@@ -1510,67 +1509,67 @@
       <c r="B14" s="1">
         <v>2458</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="6">
         <v>83</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="6">
         <v>1190000</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="6">
         <v>9.5999999999999992E-3</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="6">
         <v>5.5999999999999994E-2</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="6">
         <v>490.58</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="6">
         <v>96</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="6">
         <v>86</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="6">
         <v>60</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="6">
         <v>61</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="6">
         <v>65</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="6">
         <v>39</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="6">
         <v>33</v>
       </c>
-      <c r="O14" s="2">
+      <c r="O14" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q14">
+      <c r="Q14" s="6">
         <v>78</v>
       </c>
-      <c r="R14" s="3">
+      <c r="R14" s="6">
         <v>133.94</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="6">
         <v>0.05</v>
       </c>
-      <c r="T14">
+      <c r="T14" s="6">
         <v>48</v>
       </c>
-      <c r="U14">
+      <c r="U14" s="6">
         <v>75</v>
       </c>
-      <c r="V14" s="2">
+      <c r="V14" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W14">
+      <c r="W14" s="6">
         <v>53</v>
       </c>
     </row>
@@ -1581,67 +1580,67 @@
       <c r="B15" s="1">
         <v>2457</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="6">
         <v>75</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="6">
         <v>802900</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="6">
         <v>1.1200000000000002E-2</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="6">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="6">
         <v>252.08</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="6">
         <v>81</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="6">
         <v>65</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="6">
         <v>57</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="6">
         <v>69</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="6">
         <v>44</v>
       </c>
-      <c r="M15">
+      <c r="M15" s="6">
         <v>22</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="6">
         <v>12</v>
       </c>
-      <c r="O15" s="2">
+      <c r="O15" s="6">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="6">
         <v>9.1000000000000004E-3</v>
       </c>
-      <c r="Q15">
+      <c r="Q15" s="6">
         <v>71</v>
       </c>
-      <c r="R15" s="3">
+      <c r="R15" s="6">
         <v>120.62</v>
       </c>
-      <c r="S15" s="2">
+      <c r="S15" s="6">
         <v>0.05</v>
       </c>
-      <c r="T15">
+      <c r="T15" s="6">
         <v>39</v>
       </c>
-      <c r="U15">
+      <c r="U15" s="6">
         <v>65</v>
       </c>
-      <c r="V15" s="2">
+      <c r="V15" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W15">
+      <c r="W15" s="6">
         <v>81</v>
       </c>
     </row>
@@ -1652,67 +1651,67 @@
       <c r="B16" s="1">
         <v>2481</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="6">
         <v>80</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="6">
         <v>1840000</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="6">
         <v>1.1200000000000002E-2</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="6">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="6">
         <v>568.53</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="6">
         <v>95</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="6">
         <v>77</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="6">
         <v>58</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="6">
         <v>67</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="6">
         <v>55</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="6">
         <v>40</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="6">
         <v>32</v>
       </c>
-      <c r="O16" s="2">
+      <c r="O16" s="6">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="6">
         <v>9.1000000000000004E-3</v>
       </c>
-      <c r="Q16">
+      <c r="Q16" s="6">
         <v>76</v>
       </c>
-      <c r="R16" s="3">
+      <c r="R16" s="6">
         <v>250</v>
       </c>
-      <c r="S16" s="2">
+      <c r="S16" s="6">
         <v>0.05</v>
       </c>
-      <c r="T16">
+      <c r="T16" s="6">
         <v>43</v>
       </c>
-      <c r="U16">
+      <c r="U16" s="6">
         <v>90</v>
       </c>
-      <c r="V16" s="2">
+      <c r="V16" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W16">
+      <c r="W16" s="6">
         <v>75</v>
       </c>
     </row>
@@ -1723,67 +1722,67 @@
       <c r="B17" s="1">
         <v>2482</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="6">
         <v>81</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="6">
         <v>1470000</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="6">
         <v>1.1200000000000002E-2</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="6">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="6">
         <v>618.82000000000005</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="6">
         <v>95</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="6">
         <v>72</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="6">
         <v>58</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="6">
         <v>68</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="6">
         <v>55</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="6">
         <v>45</v>
       </c>
-      <c r="N17">
+      <c r="N17" s="6">
         <v>32</v>
       </c>
-      <c r="O17" s="2">
+      <c r="O17" s="6">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="6">
         <v>9.1000000000000004E-3</v>
       </c>
-      <c r="Q17">
+      <c r="Q17" s="6">
         <v>73</v>
       </c>
-      <c r="R17" s="3">
+      <c r="R17" s="6">
         <v>230.63</v>
       </c>
-      <c r="S17" s="2">
+      <c r="S17" s="6">
         <v>0.05</v>
       </c>
-      <c r="T17">
+      <c r="T17" s="6">
         <v>44</v>
       </c>
-      <c r="U17">
+      <c r="U17" s="6">
         <v>80</v>
       </c>
-      <c r="V17" s="2">
+      <c r="V17" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W17">
+      <c r="W17" s="6">
         <v>77</v>
       </c>
     </row>
@@ -1794,67 +1793,67 @@
       <c r="B18" s="1">
         <v>2493</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="6">
         <v>80</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="6">
         <v>2190000</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="6">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18" s="6">
         <v>0.10099999999999999</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="6">
         <v>611.70000000000005</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="6">
         <v>96</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="6">
         <v>74</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="6">
         <v>59</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="6">
         <v>71</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="6">
         <v>63</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="6">
         <v>27</v>
       </c>
-      <c r="N18">
+      <c r="N18" s="6">
         <v>27</v>
       </c>
-      <c r="O18" s="2">
+      <c r="O18" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="6">
         <v>8.6E-3</v>
       </c>
-      <c r="Q18">
+      <c r="Q18" s="6">
         <v>79</v>
       </c>
-      <c r="R18" s="3">
+      <c r="R18" s="6">
         <v>250</v>
       </c>
-      <c r="S18" s="2">
+      <c r="S18" s="6">
         <v>0.05</v>
       </c>
-      <c r="T18">
+      <c r="T18" s="6">
         <v>44</v>
       </c>
-      <c r="U18">
+      <c r="U18" s="6">
         <v>92</v>
       </c>
-      <c r="V18" s="2">
+      <c r="V18" s="6">
         <v>6.25E-2</v>
       </c>
-      <c r="W18">
+      <c r="W18" s="6">
         <v>60</v>
       </c>
     </row>

</xml_diff>

<commit_message>
changed everthing so that i can use google sheets instead of loading data
</commit_message>
<xml_diff>
--- a/data/raw/town_scores.xlsx
+++ b/data/raw/town_scores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/russ_the_bus/Desktop/Bubble_Move_Meter/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012B9334-CBE8-8347-A57D-BA630F1FBA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52BBC4AF-9C34-5D48-AC01-2C1478699CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{11A6349F-FCD6-4A46-9216-B6FF8C3D0BBE}"/>
   </bookViews>
@@ -207,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -215,6 +215,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,7 +649,7 @@
       <c r="W1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="5"/>
+      <c r="Z1" s="7"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A2" t="s">

</xml_diff>